<commit_message>
Update population group data for Uzbekistan
</commit_message>
<xml_diff>
--- a/uzbekistan_pop_grp.xlsx
+++ b/uzbekistan_pop_grp.xlsx
@@ -8,25 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/timursabitov/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CA35ED21-4636-F84B-858D-57EF7B153359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{FFF9E878-791A-024A-A85C-7C841359B262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11300" yWindow="1440" windowWidth="18100" windowHeight="15360" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16480" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Population Data" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="3" r:id="rId2"/>
     <sheet name="Sources" sheetId="2" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.4" hidden="1">Sheet1!$B$23</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">Sheet1!$B$24</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">Sheet1!$C$23:$J$23</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">Sheet1!$C$24:$J$24</definedName>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$B$23</definedName>
-    <definedName name="_xlchart.v2.1" hidden="1">Sheet1!$B$24</definedName>
-    <definedName name="_xlchart.v2.2" hidden="1">Sheet1!$C$23:$J$23</definedName>
-    <definedName name="_xlchart.v2.3" hidden="1">Sheet1!$C$24:$J$24</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -44,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="231" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="85">
   <si>
     <t>Uzbekistan Population by Region (2024–2025)</t>
   </si>
@@ -259,16 +249,10 @@
     <t>18.7% 32%</t>
   </si>
   <si>
-    <t>Population</t>
-  </si>
-  <si>
     <t>Total+unallocated</t>
   </si>
   <si>
     <t>GDP/Year</t>
-  </si>
-  <si>
-    <t>GRP (Jan-Sep)</t>
   </si>
   <si>
     <t>Jan-Dec</t>
@@ -288,6 +272,24 @@
   <si>
     <t>GDP per Capita*</t>
   </si>
+  <si>
+    <t xml:space="preserve">City population </t>
+  </si>
+  <si>
+    <t>Regions population</t>
+  </si>
+  <si>
+    <t>GDP Volume (bil sum)</t>
+  </si>
+  <si>
+    <t>Agriculture</t>
+  </si>
+  <si>
+    <t>Services</t>
+  </si>
+  <si>
+    <t>https://stat.uz/en/quarterly-reports/5870-2018#january-september</t>
+  </si>
 </sst>
 </file>
 
@@ -295,7 +297,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="#,##0.0"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -427,7 +429,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
@@ -449,15 +451,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="169" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3838,7 +3838,7 @@
         <v>5.8</v>
       </c>
       <c r="F4" s="7">
-        <f t="shared" ref="F3:F16" si="0">(((E4*100)/$E$18))*$A$19/100</f>
+        <f t="shared" ref="F4:F16" si="0">(((E4*100)/$E$18))*$A$19/100</f>
         <v>3102.5327014218014</v>
       </c>
       <c r="G4" s="7" t="s">
@@ -5745,35 +5745,35 @@
     <col min="13" max="13" width="20.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="2:21" x14ac:dyDescent="0.2">
       <c r="C1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="H1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I1" s="18" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J1" s="18" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A2" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B2" s="18" t="s">
+        <v>81</v>
       </c>
       <c r="C2" s="18">
         <v>2017</v>
@@ -5799,34 +5799,9 @@
       <c r="J2" s="18">
         <v>2024</v>
       </c>
-      <c r="N2" s="18">
-        <v>2017</v>
-      </c>
-      <c r="O2" s="18">
-        <v>2018</v>
-      </c>
-      <c r="P2" s="18">
-        <v>2019</v>
-      </c>
-      <c r="Q2" s="18">
-        <v>2020</v>
-      </c>
-      <c r="R2" s="18">
-        <v>2021</v>
-      </c>
-      <c r="S2" s="18">
-        <v>2022</v>
-      </c>
-      <c r="T2" s="18">
-        <v>2023</v>
-      </c>
-      <c r="U2" s="18">
-        <v>2024</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A3" s="24"/>
-      <c r="B3" s="25" t="s">
+    </row>
+    <row r="3" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B3" s="7" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="20">
@@ -5853,13 +5828,36 @@
       <c r="J3" s="14">
         <v>45658.5</v>
       </c>
-      <c r="M3" s="7" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A4" s="24"/>
-      <c r="B4" s="25" t="s">
+      <c r="M3" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="N3" s="18">
+        <v>2017</v>
+      </c>
+      <c r="O3" s="18">
+        <v>2018</v>
+      </c>
+      <c r="P3" s="18">
+        <v>2019</v>
+      </c>
+      <c r="Q3" s="18">
+        <v>2020</v>
+      </c>
+      <c r="R3" s="18">
+        <v>2021</v>
+      </c>
+      <c r="S3" s="18">
+        <v>2022</v>
+      </c>
+      <c r="T3" s="18">
+        <v>2023</v>
+      </c>
+      <c r="U3" s="18">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="4" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B4" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C4" s="20">
@@ -5887,12 +5885,35 @@
         <v>90522.1</v>
       </c>
       <c r="M4" s="7" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A5" s="24"/>
-      <c r="B5" s="25" t="s">
+        <v>3</v>
+      </c>
+      <c r="N4">
+        <v>15.2</v>
+      </c>
+      <c r="O4">
+        <v>27.8</v>
+      </c>
+      <c r="P4">
+        <v>28.1</v>
+      </c>
+      <c r="Q4">
+        <v>29.6</v>
+      </c>
+      <c r="R4">
+        <v>29.4</v>
+      </c>
+      <c r="S4">
+        <v>24.9</v>
+      </c>
+      <c r="T4">
+        <v>25.2</v>
+      </c>
+      <c r="U4">
+        <v>23.5</v>
+      </c>
+    </row>
+    <row r="5" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B5" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C5" s="20">
@@ -5920,12 +5941,35 @@
         <v>71560.399999999994</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A6" s="24"/>
-      <c r="B6" s="25" t="s">
+        <v>4</v>
+      </c>
+      <c r="N5">
+        <v>33.4</v>
+      </c>
+      <c r="O5">
+        <v>44.7</v>
+      </c>
+      <c r="P5">
+        <v>43.2</v>
+      </c>
+      <c r="Q5">
+        <v>42.7</v>
+      </c>
+      <c r="R5">
+        <v>43.3</v>
+      </c>
+      <c r="S5">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="T5">
+        <v>33.299999999999997</v>
+      </c>
+      <c r="U5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="20">
@@ -5953,12 +5997,35 @@
         <v>43057.9</v>
       </c>
       <c r="M6" s="7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A7" s="24"/>
-      <c r="B7" s="25" t="s">
+        <v>5</v>
+      </c>
+      <c r="N6">
+        <v>31</v>
+      </c>
+      <c r="O6">
+        <v>48.7</v>
+      </c>
+      <c r="P6">
+        <v>43.2</v>
+      </c>
+      <c r="Q6">
+        <v>46.2</v>
+      </c>
+      <c r="R6">
+        <v>45.5</v>
+      </c>
+      <c r="S6">
+        <v>39.1</v>
+      </c>
+      <c r="T6">
+        <v>37.4</v>
+      </c>
+      <c r="U6">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B7" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C7" s="20">
@@ -5986,12 +6053,35 @@
         <v>80658.3</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A8" s="24"/>
-      <c r="B8" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="N7">
+        <v>35.200000000000003</v>
+      </c>
+      <c r="O7">
+        <v>55.7</v>
+      </c>
+      <c r="P7">
+        <v>53.2</v>
+      </c>
+      <c r="Q7">
+        <v>53.8</v>
+      </c>
+      <c r="R7">
+        <v>53.5</v>
+      </c>
+      <c r="S7">
+        <v>47</v>
+      </c>
+      <c r="T7">
+        <v>43.3</v>
+      </c>
+      <c r="U7">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="8" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B8" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="20">
@@ -6019,12 +6109,35 @@
         <v>117297.8</v>
       </c>
       <c r="M8" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A9" s="24"/>
-      <c r="B9" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="N8">
+        <v>22.6</v>
+      </c>
+      <c r="O8">
+        <v>42.7</v>
+      </c>
+      <c r="P8">
+        <v>41.1</v>
+      </c>
+      <c r="Q8">
+        <v>42.4</v>
+      </c>
+      <c r="R8">
+        <v>42.1</v>
+      </c>
+      <c r="S8">
+        <v>35.5</v>
+      </c>
+      <c r="T8">
+        <v>34.6</v>
+      </c>
+      <c r="U8">
+        <v>32.700000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B9" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C9" s="20">
@@ -6052,12 +6165,35 @@
         <v>68915.7</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A10" s="24"/>
-      <c r="B10" s="25" t="s">
+        <v>8</v>
+      </c>
+      <c r="N9">
+        <v>18.5</v>
+      </c>
+      <c r="O9">
+        <v>23.1</v>
+      </c>
+      <c r="P9">
+        <v>16.3</v>
+      </c>
+      <c r="Q9">
+        <v>14</v>
+      </c>
+      <c r="R9">
+        <v>14.9</v>
+      </c>
+      <c r="S9">
+        <v>13.2</v>
+      </c>
+      <c r="T9">
+        <v>13</v>
+      </c>
+      <c r="U9">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="10" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B10" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C10" s="20">
@@ -6085,12 +6221,35 @@
         <v>99866.1</v>
       </c>
       <c r="M10" s="7" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A11" s="24"/>
-      <c r="B11" s="25" t="s">
+        <v>9</v>
+      </c>
+      <c r="N10">
+        <v>30.9</v>
+      </c>
+      <c r="O10">
+        <v>45.5</v>
+      </c>
+      <c r="P10">
+        <v>43.2</v>
+      </c>
+      <c r="Q10">
+        <v>42.4</v>
+      </c>
+      <c r="R10">
+        <v>41.4</v>
+      </c>
+      <c r="S10">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="T10">
+        <v>32.5</v>
+      </c>
+      <c r="U10">
+        <v>29.8</v>
+      </c>
+    </row>
+    <row r="11" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B11" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C11" s="20">
@@ -6118,12 +6277,35 @@
         <v>54354.1</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A12" s="24"/>
-      <c r="B12" s="25" t="s">
+        <v>10</v>
+      </c>
+      <c r="N11">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="O11">
+        <v>47.6</v>
+      </c>
+      <c r="P11">
+        <v>44.8</v>
+      </c>
+      <c r="Q11">
+        <v>45.7</v>
+      </c>
+      <c r="R11">
+        <v>43.8</v>
+      </c>
+      <c r="S11">
+        <v>35.1</v>
+      </c>
+      <c r="T11">
+        <v>34.700000000000003</v>
+      </c>
+      <c r="U11">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="12" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B12" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C12" s="20">
@@ -6151,12 +6333,35 @@
         <v>28003.3</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A13" s="24"/>
-      <c r="B13" s="25" t="s">
+        <v>11</v>
+      </c>
+      <c r="N12">
+        <v>40.299999999999997</v>
+      </c>
+      <c r="O12">
+        <v>50.8</v>
+      </c>
+      <c r="P12">
+        <v>49.9</v>
+      </c>
+      <c r="Q12">
+        <v>48.5</v>
+      </c>
+      <c r="R12">
+        <v>47.6</v>
+      </c>
+      <c r="S12">
+        <v>41.6</v>
+      </c>
+      <c r="T12">
+        <v>41.6</v>
+      </c>
+      <c r="U12">
+        <v>39.1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C13" s="20">
@@ -6184,12 +6389,35 @@
         <v>146385.20000000001</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A14" s="24"/>
-      <c r="B14" s="25" t="s">
+        <v>12</v>
+      </c>
+      <c r="N13">
+        <v>36.9</v>
+      </c>
+      <c r="O13">
+        <v>43.4</v>
+      </c>
+      <c r="P13">
+        <v>41.1</v>
+      </c>
+      <c r="Q13">
+        <v>39.799999999999997</v>
+      </c>
+      <c r="R13">
+        <v>40.299999999999997</v>
+      </c>
+      <c r="S13">
+        <v>36.4</v>
+      </c>
+      <c r="T13">
+        <v>34.4</v>
+      </c>
+      <c r="U13">
+        <v>32.6</v>
+      </c>
+    </row>
+    <row r="14" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B14" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="20">
@@ -6217,12 +6445,35 @@
         <v>91333</v>
       </c>
       <c r="M14" s="7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A15" s="24"/>
-      <c r="B15" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="N14">
+        <v>23.1</v>
+      </c>
+      <c r="O14">
+        <v>29.2</v>
+      </c>
+      <c r="P14">
+        <v>24.3</v>
+      </c>
+      <c r="Q14">
+        <v>23.5</v>
+      </c>
+      <c r="R14">
+        <v>22.5</v>
+      </c>
+      <c r="S14">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="T14">
+        <v>19.8</v>
+      </c>
+      <c r="U14">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="15" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B15" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C15" s="20">
@@ -6250,12 +6501,35 @@
         <v>51261</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="A16" s="24"/>
-      <c r="B16" s="25" t="s">
+        <v>14</v>
+      </c>
+      <c r="N15">
+        <v>23.4</v>
+      </c>
+      <c r="O15">
+        <v>39.1</v>
+      </c>
+      <c r="P15">
+        <v>35.200000000000003</v>
+      </c>
+      <c r="Q15">
+        <v>34.9</v>
+      </c>
+      <c r="R15">
+        <v>35</v>
+      </c>
+      <c r="S15">
+        <v>30.5</v>
+      </c>
+      <c r="T15">
+        <v>29.7</v>
+      </c>
+      <c r="U15">
+        <v>28.2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:21" x14ac:dyDescent="0.2">
+      <c r="B16" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C16" s="20">
@@ -6283,77 +6557,103 @@
         <v>281147.40000000002</v>
       </c>
       <c r="M16" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N16">
+        <v>30.4</v>
+      </c>
+      <c r="O16">
+        <v>48.4</v>
+      </c>
+      <c r="P16">
+        <v>46</v>
+      </c>
+      <c r="Q16">
+        <v>47.3</v>
+      </c>
+      <c r="R16">
+        <v>46.1</v>
+      </c>
+      <c r="S16">
+        <v>39.4</v>
+      </c>
+      <c r="T16">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="U16">
+        <v>34.799999999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="B17" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C17">
+        <f t="shared" ref="C17:J17" si="0">SUM(C3:C16)</f>
+        <v>252035.10000000003</v>
+      </c>
+      <c r="D17">
+        <f t="shared" si="0"/>
+        <v>351725.10000000003</v>
+      </c>
+      <c r="E17">
+        <f t="shared" si="0"/>
+        <v>453417.69999999995</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="0"/>
+        <v>521080.79999999993</v>
+      </c>
+      <c r="G17">
+        <f t="shared" si="0"/>
+        <v>648912.10000000009</v>
+      </c>
+      <c r="H17">
+        <f t="shared" si="0"/>
+        <v>865769.2</v>
+      </c>
+      <c r="I17">
+        <f t="shared" si="0"/>
+        <v>1042535.5</v>
+      </c>
+      <c r="J17">
+        <f t="shared" si="0"/>
+        <v>1270020.8000000003</v>
+      </c>
+      <c r="M17" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="N16" s="20">
-        <v>40720.400000000001</v>
-      </c>
-      <c r="O16" s="20">
-        <v>63509.2</v>
-      </c>
-      <c r="P16" s="19">
-        <v>84720.4</v>
-      </c>
-      <c r="Q16" s="19">
-        <v>95247.8</v>
-      </c>
-      <c r="R16" s="19">
-        <v>121779.8</v>
-      </c>
-      <c r="S16" s="19">
-        <v>172469.3</v>
-      </c>
-      <c r="T16" s="19">
-        <v>215099.2</v>
-      </c>
-      <c r="U16" s="23">
-        <v>281147.40000000002</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A17" s="24"/>
-      <c r="B17" s="25" t="s">
-        <v>48</v>
-      </c>
-      <c r="C17" s="24">
-        <f>SUM(C3:C16)</f>
-        <v>252035.10000000003</v>
-      </c>
-      <c r="D17" s="24">
-        <f>SUM(D3:D16)</f>
-        <v>351725.10000000003</v>
-      </c>
-      <c r="E17" s="24">
-        <f>SUM(E3:E16)</f>
-        <v>453417.69999999995</v>
-      </c>
-      <c r="F17" s="24">
-        <f>SUM(F3:F16)</f>
-        <v>521080.79999999993</v>
-      </c>
-      <c r="G17" s="24">
-        <f>SUM(G3:G16)</f>
-        <v>648912.10000000009</v>
-      </c>
-      <c r="H17" s="24">
-        <f>SUM(H3:H16)</f>
-        <v>865769.2</v>
-      </c>
-      <c r="I17" s="24">
-        <f>SUM(I3:I16)</f>
-        <v>1042535.5</v>
-      </c>
-      <c r="J17" s="24">
-        <f>SUM(J3:J16)</f>
-        <v>1270020.8000000003</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>0</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>0</v>
+      </c>
+      <c r="U17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A18" s="18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C18" s="21">
         <v>356453.84090000001</v>
@@ -6380,9 +6680,9 @@
         <v>1454573.8673999999</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A19" s="18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C19" s="19">
         <v>5113</v>
@@ -6409,9 +6709,9 @@
         <v>12652</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A20" s="10" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C20" s="18">
         <f>C18/C19</f>
@@ -6422,33 +6722,33 @@
         <v>58.627651120188141</v>
       </c>
       <c r="E20" s="18">
-        <f t="shared" ref="E20:J20" si="0">E18/E19</f>
+        <f t="shared" ref="E20:J20" si="1">E18/E19</f>
         <v>67.414079469447913</v>
       </c>
       <c r="F20" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>66.617267092142001</v>
       </c>
       <c r="G20" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>77.31429497785733</v>
       </c>
       <c r="H20" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90.08080804379297</v>
       </c>
       <c r="I20" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>102.57049773482072</v>
       </c>
       <c r="J20" s="18">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>114.96789973126778</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B23" s="18" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C23" s="18">
         <v>2017</v>
@@ -6474,8 +6774,35 @@
       <c r="J23" s="18">
         <v>2024</v>
       </c>
-    </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M23" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="N23" s="18">
+        <v>2017</v>
+      </c>
+      <c r="O23" s="18">
+        <v>2018</v>
+      </c>
+      <c r="P23" s="18">
+        <v>2019</v>
+      </c>
+      <c r="Q23" s="18">
+        <v>2020</v>
+      </c>
+      <c r="R23" s="18">
+        <v>2021</v>
+      </c>
+      <c r="S23" s="18">
+        <v>2022</v>
+      </c>
+      <c r="T23" s="18">
+        <v>2023</v>
+      </c>
+      <c r="U23" s="18">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B24" s="7" t="s">
         <v>3</v>
       </c>
@@ -6484,523 +6811,901 @@
         <v>1558.9034981724869</v>
       </c>
       <c r="D24" s="14">
-        <f t="shared" ref="D24:J24" si="1">(D$18/D$17)*(D3/D$19)/D44*1000000</f>
+        <f t="shared" ref="D24:J24" si="2">(D$18/D$17)*(D3/D$19)/D44*1000000</f>
         <v>1413.4878969382414</v>
       </c>
       <c r="E24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1555.1032154998952</v>
       </c>
       <c r="F24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1458.8594060936991</v>
       </c>
       <c r="G24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1590.6038970010447</v>
       </c>
       <c r="H24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1897.8710727214789</v>
       </c>
       <c r="I24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>1949.8991636011572</v>
       </c>
       <c r="J24" s="14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>2063.8185218166236</v>
       </c>
-    </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M24" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N24">
+        <v>32.700000000000003</v>
+      </c>
+      <c r="O24">
+        <v>30</v>
+      </c>
+      <c r="P24">
+        <v>28.1</v>
+      </c>
+      <c r="Q24">
+        <v>26.4</v>
+      </c>
+      <c r="R24">
+        <v>25.6</v>
+      </c>
+      <c r="S24">
+        <v>21.5</v>
+      </c>
+      <c r="T24">
+        <v>20</v>
+      </c>
+      <c r="U24">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B25" s="7" t="s">
         <v>4</v>
       </c>
       <c r="C25" s="14">
-        <f t="shared" ref="C25:J25" si="2">(C$18/C$17)*(C4/C$19)/C45*1000000</f>
+        <f t="shared" ref="C25:J25" si="3">(C$18/C$17)*(C4/C$19)/C45*1000000</f>
         <v>1793.2673606015076</v>
       </c>
       <c r="D25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1495.3257053552124</v>
       </c>
       <c r="E25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1627.9836093962751</v>
       </c>
       <c r="F25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1553.5934495743256</v>
       </c>
       <c r="G25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>1619.4059774803452</v>
       </c>
       <c r="H25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2014.1492122298459</v>
       </c>
       <c r="I25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2289.986143424504</v>
       </c>
       <c r="J25" s="14">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>2414.1117262796542</v>
       </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M25" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N25">
+        <v>20.8</v>
+      </c>
+      <c r="O25">
+        <v>22.4</v>
+      </c>
+      <c r="P25">
+        <v>23.6</v>
+      </c>
+      <c r="Q25">
+        <v>22.9</v>
+      </c>
+      <c r="R25">
+        <v>20.100000000000001</v>
+      </c>
+      <c r="S25">
+        <v>23.9</v>
+      </c>
+      <c r="T25">
+        <v>27.8</v>
+      </c>
+      <c r="U25">
+        <v>28.8</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B26" s="7" t="s">
         <v>5</v>
       </c>
       <c r="C26" s="14">
-        <f t="shared" ref="C26:J26" si="3">(C$18/C$17)*(C5/C$19)/C46*1000000</f>
+        <f t="shared" ref="C26:J26" si="4">(C$18/C$17)*(C5/C$19)/C46*1000000</f>
         <v>2476.3980064145239</v>
       </c>
       <c r="D26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>1944.5274327511358</v>
       </c>
       <c r="E26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2194.197075531486</v>
       </c>
       <c r="F26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2082.1780191302905</v>
       </c>
       <c r="G26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2346.6708118097863</v>
       </c>
       <c r="H26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2722.6580287452334</v>
       </c>
       <c r="I26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>2998.1544249936396</v>
       </c>
       <c r="J26" s="14">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3169.2582670540764</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M26" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="N26">
+        <v>19.7</v>
+      </c>
+      <c r="O26">
+        <v>12.9</v>
+      </c>
+      <c r="P26">
+        <v>19</v>
+      </c>
+      <c r="Q26">
+        <v>16.8</v>
+      </c>
+      <c r="R26">
+        <v>16.5</v>
+      </c>
+      <c r="S26">
+        <v>17.399999999999999</v>
+      </c>
+      <c r="T26">
+        <v>19.100000000000001</v>
+      </c>
+      <c r="U26">
+        <v>19.899999999999999</v>
+      </c>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B27" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C27" s="14">
-        <f t="shared" ref="C27:J27" si="4">(C$18/C$17)*(C6/C$19)/C47*1000000</f>
+        <f t="shared" ref="C27:J27" si="5">(C$18/C$17)*(C6/C$19)/C47*1000000</f>
         <v>1945.0021475861897</v>
       </c>
       <c r="D27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1599.6321067356387</v>
       </c>
       <c r="E27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1765.1720465693713</v>
       </c>
       <c r="F27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1705.859376054588</v>
       </c>
       <c r="G27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>1965.9726197128794</v>
       </c>
       <c r="H27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2188.9978254300713</v>
       </c>
       <c r="I27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2492.6934416506879</v>
       </c>
       <c r="J27" s="14">
-        <f t="shared" si="4"/>
+        <f t="shared" si="5"/>
         <v>2585.7712219585069</v>
       </c>
-    </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="N27">
+        <v>14.3</v>
+      </c>
+      <c r="O27">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="P27">
+        <v>10.1</v>
+      </c>
+      <c r="Q27">
+        <v>11.1</v>
+      </c>
+      <c r="R27">
+        <v>12.2</v>
+      </c>
+      <c r="S27">
+        <v>13.4</v>
+      </c>
+      <c r="T27">
+        <v>16.600000000000001</v>
+      </c>
+      <c r="U27">
+        <v>17.3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B28" s="7" t="s">
         <v>7</v>
       </c>
       <c r="C28" s="14">
-        <f t="shared" ref="C28:J28" si="5">(C$18/C$17)*(C7/C$19)/C48*1000000</f>
+        <f t="shared" ref="C28:J28" si="6">(C$18/C$17)*(C7/C$19)/C48*1000000</f>
         <v>2026.8727717737411</v>
       </c>
       <c r="D28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1399.7568822911689</v>
       </c>
       <c r="E28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1491.0557031778328</v>
       </c>
       <c r="F28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1377.7257763165551</v>
       </c>
       <c r="G28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1520.3012875800346</v>
       </c>
       <c r="H28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1759.2767542378567</v>
       </c>
       <c r="I28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>1939.532729116341</v>
       </c>
       <c r="J28" s="14">
-        <f t="shared" si="5"/>
+        <f t="shared" si="6"/>
         <v>2050.6504642756436</v>
       </c>
-    </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M28" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N28">
+        <v>35.200000000000003</v>
+      </c>
+      <c r="O28">
+        <v>17.7</v>
+      </c>
+      <c r="P28">
+        <v>17.8</v>
+      </c>
+      <c r="Q28">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="R28">
+        <v>17</v>
+      </c>
+      <c r="S28">
+        <v>16.5</v>
+      </c>
+      <c r="T28">
+        <v>16.8</v>
+      </c>
+      <c r="U28">
+        <v>17.7</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B29" s="7" t="s">
         <v>8</v>
       </c>
       <c r="C29" s="14">
-        <f t="shared" ref="C29:J29" si="6">(C$18/C$17)*(C8/C$19)/C49*1000000</f>
+        <f t="shared" ref="C29:J29" si="7">(C$18/C$17)*(C8/C$19)/C49*1000000</f>
         <v>4175.6005168445727</v>
       </c>
       <c r="D29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>3927.612896136347</v>
       </c>
       <c r="E29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>5498.5439485723437</v>
       </c>
       <c r="F29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>6382.6555355449027</v>
       </c>
       <c r="G29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>6903.5034304091896</v>
       </c>
       <c r="H29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>7245.1688838834689</v>
       </c>
       <c r="I29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>8222.7631460062767</v>
       </c>
       <c r="J29" s="14">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>9874.747166791929</v>
       </c>
-    </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M29" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N29">
+        <v>53.9</v>
+      </c>
+      <c r="O29">
+        <v>54.6</v>
+      </c>
+      <c r="P29">
+        <v>65.2</v>
+      </c>
+      <c r="Q29">
+        <v>70.900000000000006</v>
+      </c>
+      <c r="R29">
+        <v>69</v>
+      </c>
+      <c r="S29">
+        <v>67.8</v>
+      </c>
+      <c r="T29">
+        <v>68.400000000000006</v>
+      </c>
+      <c r="U29">
+        <v>72.099999999999994</v>
+      </c>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B30" s="7" t="s">
         <v>9</v>
       </c>
       <c r="C30" s="14">
-        <f t="shared" ref="C30:J30" si="7">(C$18/C$17)*(C9/C$19)/C50*1000000</f>
+        <f t="shared" ref="C30:J30" si="8">(C$18/C$17)*(C9/C$19)/C50*1000000</f>
         <v>1512.2771896089218</v>
       </c>
       <c r="D30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1161.3931858463741</v>
       </c>
       <c r="E30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1283.4567753923004</v>
       </c>
       <c r="F30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1267.3006892411047</v>
       </c>
       <c r="G30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1707.6281374904838</v>
       </c>
       <c r="H30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1722.1219587410842</v>
       </c>
       <c r="I30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>1909.4096179788285</v>
       </c>
       <c r="J30" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" si="8"/>
         <v>2034.6870477661403</v>
       </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M30" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="N30">
+        <v>14.9</v>
+      </c>
+      <c r="O30">
+        <v>12.6</v>
+      </c>
+      <c r="P30">
+        <v>12.7</v>
+      </c>
+      <c r="Q30">
+        <v>13.7</v>
+      </c>
+      <c r="R30">
+        <v>14.6</v>
+      </c>
+      <c r="S30">
+        <v>13.9</v>
+      </c>
+      <c r="T30">
+        <v>15.1</v>
+      </c>
+      <c r="U30">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B31" s="7" t="s">
         <v>10</v>
       </c>
       <c r="C31" s="14">
-        <f t="shared" ref="C31:J31" si="8">(C$18/C$17)*(C10/C$19)/C51*1000000</f>
+        <f t="shared" ref="C31:J31" si="9">(C$18/C$17)*(C10/C$19)/C51*1000000</f>
         <v>1936.862175533475</v>
       </c>
       <c r="D31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1464.3643849782807</v>
       </c>
       <c r="E31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1517.2045923677015</v>
       </c>
       <c r="F31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1418.5473749752528</v>
       </c>
       <c r="G31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1596.3676288292686</v>
       </c>
       <c r="H31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1780.5835421953993</v>
       </c>
       <c r="I31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>1986.4782688406128</v>
       </c>
       <c r="J31" s="14">
-        <f t="shared" si="8"/>
+        <f t="shared" si="9"/>
         <v>2148.1100271712821</v>
       </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M31" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="N31">
+        <v>18.600000000000001</v>
+      </c>
+      <c r="O31">
+        <v>14.7</v>
+      </c>
+      <c r="P31">
+        <v>13.8</v>
+      </c>
+      <c r="Q31">
+        <v>14.7</v>
+      </c>
+      <c r="R31">
+        <v>14.2</v>
+      </c>
+      <c r="S31">
+        <v>15.9</v>
+      </c>
+      <c r="T31">
+        <v>15.6</v>
+      </c>
+      <c r="U31">
+        <v>16.7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B32" s="7" t="s">
         <v>11</v>
       </c>
       <c r="C32" s="14">
-        <f t="shared" ref="C32:J32" si="9">(C$18/C$17)*(C11/C$19)/C52*1000000</f>
+        <f t="shared" ref="C32:J32" si="10">(C$18/C$17)*(C11/C$19)/C52*1000000</f>
         <v>1539.2735813187867</v>
       </c>
       <c r="D32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1232.642396480361</v>
       </c>
       <c r="E32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1289.4632296366331</v>
       </c>
       <c r="F32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1197.4612173503103</v>
       </c>
       <c r="G32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1319.6735621178859</v>
       </c>
       <c r="H32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1486.8894438270841</v>
       </c>
       <c r="I32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1647.6199037884928</v>
       </c>
       <c r="J32" s="14">
-        <f t="shared" si="9"/>
+        <f t="shared" si="10"/>
         <v>1710.1850904150283</v>
       </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M32" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="N32">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="O32">
+        <v>6.6</v>
+      </c>
+      <c r="P32">
+        <v>6.5</v>
+      </c>
+      <c r="Q32">
+        <v>7</v>
+      </c>
+      <c r="R32">
+        <v>7.3</v>
+      </c>
+      <c r="S32">
+        <v>7.3</v>
+      </c>
+      <c r="T32">
+        <v>8.1</v>
+      </c>
+      <c r="U32">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B33" s="7" t="s">
         <v>12</v>
       </c>
       <c r="C33" s="14">
-        <f t="shared" ref="C33:J33" si="10">(C$18/C$17)*(C12/C$19)/C53*1000000</f>
+        <f t="shared" ref="C33:J33" si="11">(C$18/C$17)*(C12/C$19)/C53*1000000</f>
         <v>2215.421633294588</v>
       </c>
       <c r="D33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>1743.2058572423773</v>
       </c>
       <c r="E33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>2125.6973814510502</v>
       </c>
       <c r="F33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>1934.1772991275543</v>
       </c>
       <c r="G33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>2085.8241797004421</v>
       </c>
       <c r="H33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>2386.9024686956704</v>
       </c>
       <c r="I33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>2633.7520053098474</v>
       </c>
       <c r="J33" s="14">
-        <f t="shared" si="10"/>
+        <f t="shared" si="11"/>
         <v>2773.5039016068818</v>
       </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M33" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N33">
+        <v>24.7</v>
+      </c>
+      <c r="O33">
+        <v>21.3</v>
+      </c>
+      <c r="P33">
+        <v>24.1</v>
+      </c>
+      <c r="Q33">
+        <v>23.6</v>
+      </c>
+      <c r="R33">
+        <v>23.8</v>
+      </c>
+      <c r="S33">
+        <v>23.2</v>
+      </c>
+      <c r="T33">
+        <v>26.1</v>
+      </c>
+      <c r="U33">
+        <v>27.3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B34" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C34" s="14">
-        <f t="shared" ref="C34:J34" si="11">(C$18/C$17)*(C13/C$19)/C54*1000000</f>
+        <f t="shared" ref="C34:J34" si="12">(C$18/C$17)*(C13/C$19)/C54*1000000</f>
         <v>2722.5461548310445</v>
       </c>
       <c r="D34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2329.7066254182428</v>
       </c>
       <c r="E34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2808.9028720369943</v>
       </c>
       <c r="F34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>2798.9230017084446</v>
       </c>
       <c r="G34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3291.8692289089049</v>
       </c>
       <c r="H34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3651.9891302911674</v>
       </c>
       <c r="I34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>3991.5163533815598</v>
       </c>
       <c r="J34" s="14">
-        <f t="shared" si="11"/>
+        <f t="shared" si="12"/>
         <v>4342.1704309470588</v>
       </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M34" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N34">
+        <v>38.700000000000003</v>
+      </c>
+      <c r="O34">
+        <v>40.6</v>
+      </c>
+      <c r="P34">
+        <v>45.9</v>
+      </c>
+      <c r="Q34">
+        <v>47.6</v>
+      </c>
+      <c r="R34">
+        <v>49.2</v>
+      </c>
+      <c r="S34">
+        <v>45.5</v>
+      </c>
+      <c r="T34">
+        <v>44.3</v>
+      </c>
+      <c r="U34">
+        <v>44.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B35" s="7" t="s">
         <v>14</v>
       </c>
       <c r="C35" s="14">
-        <f t="shared" ref="C35:J35" si="12">(C$18/C$17)*(C14/C$19)/C55*1000000</f>
+        <f t="shared" ref="C35:J35" si="13">(C$18/C$17)*(C14/C$19)/C55*1000000</f>
         <v>1539.282206123567</v>
       </c>
       <c r="D35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1267.2915533958596</v>
       </c>
       <c r="E35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1312.7325880967542</v>
       </c>
       <c r="F35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1268.0925124512239</v>
       </c>
       <c r="G35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1489.6334963359204</v>
       </c>
       <c r="H35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1749.5241715918828</v>
       </c>
       <c r="I35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>1930.1771863011968</v>
       </c>
       <c r="J35" s="14">
-        <f t="shared" si="12"/>
+        <f t="shared" si="13"/>
         <v>2035.668373272789</v>
       </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M35" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="N35">
+        <v>24.6</v>
+      </c>
+      <c r="O35">
+        <v>19.600000000000001</v>
+      </c>
+      <c r="P35">
+        <v>20.6</v>
+      </c>
+      <c r="Q35">
+        <v>20.8</v>
+      </c>
+      <c r="R35">
+        <v>20.7</v>
+      </c>
+      <c r="S35">
+        <v>18.8</v>
+      </c>
+      <c r="T35">
+        <v>19.3</v>
+      </c>
+      <c r="U35">
+        <v>19.8</v>
+      </c>
+    </row>
+    <row r="36" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B36" s="7" t="s">
         <v>15</v>
       </c>
       <c r="C36" s="14">
-        <f t="shared" ref="C36:J36" si="13">(C$18/C$17)*(C15/C$19)/C56*1000000</f>
+        <f t="shared" ref="C36:J36" si="14">(C$18/C$17)*(C15/C$19)/C56*1000000</f>
         <v>1783.7372030183981</v>
       </c>
       <c r="D36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1468.3236113010753</v>
       </c>
       <c r="E36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1549.3337042529031</v>
       </c>
       <c r="F36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1459.981099787233</v>
       </c>
       <c r="G36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>1665.3859782240534</v>
       </c>
       <c r="H36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>2024.3446346801513</v>
       </c>
       <c r="I36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>2194.0530072489773</v>
       </c>
       <c r="J36" s="14">
-        <f t="shared" si="13"/>
+        <f t="shared" si="14"/>
         <v>2325.3018800328973</v>
       </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M36" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N36">
+        <v>17.3</v>
+      </c>
+      <c r="O36">
+        <v>12.8</v>
+      </c>
+      <c r="P36">
+        <v>12.4</v>
+      </c>
+      <c r="Q36">
+        <v>12.2</v>
+      </c>
+      <c r="R36">
+        <v>13</v>
+      </c>
+      <c r="S36">
+        <v>15.2</v>
+      </c>
+      <c r="T36">
+        <v>15.1</v>
+      </c>
+      <c r="U36">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B37" s="7" t="s">
         <v>16</v>
       </c>
       <c r="C37" s="14">
-        <f t="shared" ref="C37:J37" si="14">(C$18/C$17)*(C16/C$19)/C57*1000000</f>
+        <f t="shared" ref="C37:J37" si="15">(C$18/C$17)*(C16/C$19)/C57*1000000</f>
         <v>4646.5218348172457</v>
       </c>
       <c r="D37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4294.7359771626143</v>
       </c>
       <c r="E37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5018.6131250561448</v>
       </c>
       <c r="F37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>4734.9608163934499</v>
       </c>
       <c r="G37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>5385.017441306577</v>
       </c>
       <c r="H37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>6273.1375167536953</v>
       </c>
       <c r="I37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>7158.2557734097409</v>
       </c>
       <c r="J37" s="14">
-        <f t="shared" si="14"/>
+        <f t="shared" si="15"/>
         <v>8369.7402253810706</v>
       </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M37" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N37" s="20">
+        <v>32.200000000000003</v>
+      </c>
+      <c r="O37" s="20">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="P37" s="19">
+        <v>35.4</v>
+      </c>
+      <c r="Q37" s="19">
+        <v>34.5</v>
+      </c>
+      <c r="R37" s="19">
+        <v>35.1</v>
+      </c>
+      <c r="S37" s="19">
+        <v>31.2</v>
+      </c>
+      <c r="T37" s="19">
+        <v>28.2</v>
+      </c>
+      <c r="U37" s="23">
+        <v>27.8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B38" s="10" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B43" s="18" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="C43" s="18">
         <v>2017</v>
@@ -7026,8 +7731,35 @@
       <c r="J43" s="18">
         <v>2024</v>
       </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M43" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="N43" s="18">
+        <v>2017</v>
+      </c>
+      <c r="O43" s="18">
+        <v>2018</v>
+      </c>
+      <c r="P43" s="18">
+        <v>2019</v>
+      </c>
+      <c r="Q43" s="18">
+        <v>2020</v>
+      </c>
+      <c r="R43" s="18">
+        <v>2021</v>
+      </c>
+      <c r="S43" s="18">
+        <v>2022</v>
+      </c>
+      <c r="T43" s="18">
+        <v>2023</v>
+      </c>
+      <c r="U43" s="18">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="44" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>1</v>
       </c>
@@ -7058,8 +7790,35 @@
       <c r="J44">
         <v>2002.7</v>
       </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M44" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="N44">
+        <v>7.5</v>
+      </c>
+      <c r="O44">
+        <v>6.7</v>
+      </c>
+      <c r="P44">
+        <v>8.1</v>
+      </c>
+      <c r="Q44">
+        <v>8.6</v>
+      </c>
+      <c r="R44">
+        <v>8</v>
+      </c>
+      <c r="S44">
+        <v>9.3000000000000007</v>
+      </c>
+      <c r="T44">
+        <v>8.3000000000000007</v>
+      </c>
+      <c r="U44">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>2</v>
       </c>
@@ -7090,8 +7849,35 @@
       <c r="J45">
         <v>3394.4</v>
       </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M45" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="N45">
+        <v>5.6</v>
+      </c>
+      <c r="O45">
+        <v>4.8</v>
+      </c>
+      <c r="P45">
+        <v>4.8</v>
+      </c>
+      <c r="Q45">
+        <v>5.6</v>
+      </c>
+      <c r="R45">
+        <v>5.8</v>
+      </c>
+      <c r="S45">
+        <v>6.8</v>
+      </c>
+      <c r="T45">
+        <v>5.7</v>
+      </c>
+      <c r="U45">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>3</v>
       </c>
@@ -7122,8 +7908,35 @@
       <c r="J46">
         <v>2044</v>
       </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M46" s="7" t="s">
+        <v>5</v>
+      </c>
+      <c r="N46">
+        <v>9.6999999999999993</v>
+      </c>
+      <c r="O46">
+        <v>7.7</v>
+      </c>
+      <c r="P46">
+        <v>7.4</v>
+      </c>
+      <c r="Q46">
+        <v>8</v>
+      </c>
+      <c r="R46">
+        <v>8.5</v>
+      </c>
+      <c r="S46">
+        <v>10</v>
+      </c>
+      <c r="T46">
+        <v>9.5</v>
+      </c>
+      <c r="U46">
+        <v>9.9</v>
+      </c>
+    </row>
+    <row r="47" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>4</v>
       </c>
@@ -7154,8 +7967,35 @@
       <c r="J47">
         <v>1507.4</v>
       </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="M47" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="N47">
+        <v>8.1</v>
+      </c>
+      <c r="O47">
+        <v>5.7</v>
+      </c>
+      <c r="P47">
+        <v>7.2</v>
+      </c>
+      <c r="Q47">
+        <v>6.6</v>
+      </c>
+      <c r="R47">
+        <v>5.9</v>
+      </c>
+      <c r="S47">
+        <v>7</v>
+      </c>
+      <c r="T47">
+        <v>6.4</v>
+      </c>
+      <c r="U47">
+        <v>6.2</v>
+      </c>
+    </row>
+    <row r="48" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>5</v>
       </c>
@@ -7186,8 +8026,35 @@
       <c r="J48">
         <v>3560.6</v>
       </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M48" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="N48">
+        <v>7.6</v>
+      </c>
+      <c r="O48">
+        <v>6.5</v>
+      </c>
+      <c r="P48">
+        <v>6.4</v>
+      </c>
+      <c r="Q48">
+        <v>6.2</v>
+      </c>
+      <c r="R48">
+        <v>6.6</v>
+      </c>
+      <c r="S48">
+        <v>7.9</v>
+      </c>
+      <c r="T48">
+        <v>8.1</v>
+      </c>
+      <c r="U48">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>6</v>
       </c>
@@ -7218,8 +8085,35 @@
       <c r="J49">
         <v>1075.3</v>
       </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M49" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="N49">
+        <v>4.8</v>
+      </c>
+      <c r="O49">
+        <v>4.5</v>
+      </c>
+      <c r="P49">
+        <v>4.2</v>
+      </c>
+      <c r="Q49">
+        <v>3.4</v>
+      </c>
+      <c r="R49">
+        <v>3.8</v>
+      </c>
+      <c r="S49">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="T49">
+        <v>4.7</v>
+      </c>
+      <c r="U49">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>7</v>
       </c>
@@ -7250,8 +8144,35 @@
       <c r="J50">
         <v>3066.1</v>
       </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M50" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="N50">
+        <v>6.8</v>
+      </c>
+      <c r="O50">
+        <v>5.5</v>
+      </c>
+      <c r="P50">
+        <v>6.7</v>
+      </c>
+      <c r="Q50">
+        <v>7.5</v>
+      </c>
+      <c r="R50">
+        <v>7.3</v>
+      </c>
+      <c r="S50">
+        <v>8.8000000000000007</v>
+      </c>
+      <c r="T50">
+        <v>8</v>
+      </c>
+      <c r="U50">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A51">
         <v>8</v>
       </c>
@@ -7282,8 +8203,35 @@
       <c r="J51">
         <v>4208.5</v>
       </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M51" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="N51">
+        <v>5.9</v>
+      </c>
+      <c r="O51">
+        <v>4.5999999999999996</v>
+      </c>
+      <c r="P51">
+        <v>5.3</v>
+      </c>
+      <c r="Q51">
+        <v>5.9</v>
+      </c>
+      <c r="R51">
+        <v>6.1</v>
+      </c>
+      <c r="S51">
+        <v>6.5</v>
+      </c>
+      <c r="T51">
+        <v>6.2</v>
+      </c>
+      <c r="U51">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A52">
         <v>9</v>
       </c>
@@ -7314,8 +8262,35 @@
       <c r="J52">
         <v>2877.1</v>
       </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M52" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="N52">
+        <v>7.7</v>
+      </c>
+      <c r="O52">
+        <v>6.9</v>
+      </c>
+      <c r="P52">
+        <v>8</v>
+      </c>
+      <c r="Q52">
+        <v>8.6</v>
+      </c>
+      <c r="R52">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="S52">
+        <v>10.6</v>
+      </c>
+      <c r="T52">
+        <v>9.9</v>
+      </c>
+      <c r="U52">
+        <v>9.4</v>
+      </c>
+    </row>
+    <row r="53" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A53">
         <v>10</v>
       </c>
@@ -7346,8 +8321,35 @@
       <c r="J53">
         <v>914</v>
       </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M53" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="N53">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="O53">
+        <v>5.5</v>
+      </c>
+      <c r="P53">
+        <v>7.6</v>
+      </c>
+      <c r="Q53">
+        <v>8.5</v>
+      </c>
+      <c r="R53">
+        <v>7.9</v>
+      </c>
+      <c r="S53">
+        <v>8.6999999999999993</v>
+      </c>
+      <c r="T53">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="U53">
+        <v>7.6</v>
+      </c>
+    </row>
+    <row r="54" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A54">
         <v>11</v>
       </c>
@@ -7378,8 +8380,35 @@
       <c r="J54">
         <v>3051.8</v>
       </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M54" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N54">
+        <v>3.7</v>
+      </c>
+      <c r="O54">
+        <v>3.4</v>
+      </c>
+      <c r="P54">
+        <v>4.7</v>
+      </c>
+      <c r="Q54">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="R54">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="S54">
+        <v>7.1</v>
+      </c>
+      <c r="T54">
+        <v>7.2</v>
+      </c>
+      <c r="U54">
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="55" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A55">
         <v>12</v>
       </c>
@@ -7410,8 +8439,35 @@
       <c r="J55">
         <v>4061.5</v>
       </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M55" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="N55">
+        <v>6.2</v>
+      </c>
+      <c r="O55">
+        <v>5</v>
+      </c>
+      <c r="P55">
+        <v>5.9</v>
+      </c>
+      <c r="Q55">
+        <v>6.6</v>
+      </c>
+      <c r="R55">
+        <v>6.5</v>
+      </c>
+      <c r="S55">
+        <v>8</v>
+      </c>
+      <c r="T55">
+        <v>7.7</v>
+      </c>
+      <c r="U55">
+        <v>7.3</v>
+      </c>
+    </row>
+    <row r="56" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A56">
         <v>13</v>
       </c>
@@ -7442,8 +8498,35 @@
       <c r="J56">
         <v>1995.6</v>
       </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M56" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="N56">
+        <v>7.2</v>
+      </c>
+      <c r="O56">
+        <v>5.4</v>
+      </c>
+      <c r="P56">
+        <v>6</v>
+      </c>
+      <c r="Q56">
+        <v>6</v>
+      </c>
+      <c r="R56">
+        <v>7.1</v>
+      </c>
+      <c r="S56">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="T56">
+        <v>8.5</v>
+      </c>
+      <c r="U56">
+        <v>8.9</v>
+      </c>
+    </row>
+    <row r="57" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A57">
         <v>14</v>
       </c>
@@ -7474,47 +8557,74 @@
       <c r="J57">
         <v>3040.8</v>
       </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M57" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="N57" s="20">
+        <v>7.4</v>
+      </c>
+      <c r="O57" s="20">
+        <v>8.1</v>
+      </c>
+      <c r="P57" s="19">
+        <v>9.1999999999999993</v>
+      </c>
+      <c r="Q57" s="19">
+        <v>9.5</v>
+      </c>
+      <c r="R57" s="19">
+        <v>10.1</v>
+      </c>
+      <c r="S57" s="19">
+        <v>11.5</v>
+      </c>
+      <c r="T57" s="19">
+        <v>10.4</v>
+      </c>
+      <c r="U57" s="23">
+        <v>9.1999999999999993</v>
+      </c>
+    </row>
+    <row r="58" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B58" s="7" t="s">
         <v>48</v>
       </c>
       <c r="C58" s="7">
-        <f>SUM(C44:C57)</f>
+        <f t="shared" ref="C58:J58" si="16">SUM(C44:C57)</f>
         <v>32120.499999999993</v>
       </c>
       <c r="D58" s="7">
-        <f>SUM(D44:D57)</f>
+        <f t="shared" si="16"/>
         <v>32656.700000000004</v>
       </c>
       <c r="E58" s="7">
-        <f>SUM(E44:E57)</f>
+        <f t="shared" si="16"/>
         <v>33255.5</v>
       </c>
       <c r="F58" s="7">
-        <f>SUM(F44:F57)</f>
+        <f t="shared" si="16"/>
         <v>33905.199999999997</v>
       </c>
       <c r="G58" s="7">
-        <f>SUM(G44:G57)</f>
+        <f t="shared" si="16"/>
         <v>34558.9</v>
       </c>
       <c r="H58" s="7">
-        <f>SUM(H44:H57)</f>
+        <f t="shared" si="16"/>
         <v>35271.300000000003</v>
       </c>
       <c r="I58" s="7">
-        <f>SUM(I44:I57)</f>
+        <f t="shared" si="16"/>
         <v>36024.9</v>
       </c>
       <c r="J58" s="7">
-        <f>SUM(J44:J57)</f>
+        <f t="shared" si="16"/>
         <v>36799.800000000003</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B62" s="18" t="s">
-        <v>59</v>
+        <v>79</v>
       </c>
       <c r="C62" s="18">
         <v>2017</v>
@@ -7541,7 +8651,7 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A63">
         <v>1</v>
       </c>
@@ -7573,8 +8683,35 @@
         <v>480.8</v>
       </c>
       <c r="K63" s="20"/>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="M63" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="N63" s="18">
+        <v>2017</v>
+      </c>
+      <c r="O63" s="19">
+        <v>2018</v>
+      </c>
+      <c r="P63" s="19">
+        <v>2019</v>
+      </c>
+      <c r="Q63" s="19">
+        <v>2020</v>
+      </c>
+      <c r="R63" s="19">
+        <v>2021</v>
+      </c>
+      <c r="S63" s="19">
+        <v>2022</v>
+      </c>
+      <c r="T63" s="19">
+        <v>2023</v>
+      </c>
+      <c r="U63" s="19">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="64" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A64">
         <v>2</v>
       </c>
@@ -7606,8 +8743,35 @@
         <v>294.5</v>
       </c>
       <c r="K64" s="20"/>
-    </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M64" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="N64" s="14">
+        <v>44.6</v>
+      </c>
+      <c r="O64" s="20">
+        <v>35.5</v>
+      </c>
+      <c r="P64" s="20">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="Q64" s="20">
+        <v>35.4</v>
+      </c>
+      <c r="R64" s="20">
+        <v>37</v>
+      </c>
+      <c r="S64" s="20">
+        <v>44.3</v>
+      </c>
+      <c r="T64" s="20">
+        <v>46.5</v>
+      </c>
+      <c r="U64" s="20">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="65" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A65">
         <v>3</v>
       </c>
@@ -7639,8 +8803,35 @@
         <v>195.8</v>
       </c>
       <c r="K65" s="20"/>
-    </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M65" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="N65" s="20">
+        <v>40.200000000000003</v>
+      </c>
+      <c r="O65" s="20">
+        <v>28.1</v>
+      </c>
+      <c r="P65" s="20">
+        <v>28.4</v>
+      </c>
+      <c r="Q65" s="20">
+        <v>28.8</v>
+      </c>
+      <c r="R65" s="20">
+        <v>30.8</v>
+      </c>
+      <c r="S65" s="20">
+        <v>33.6</v>
+      </c>
+      <c r="T65" s="20">
+        <v>33.200000000000003</v>
+      </c>
+      <c r="U65" s="20">
+        <v>34.299999999999997</v>
+      </c>
+    </row>
+    <row r="66" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A66">
         <v>4</v>
       </c>
@@ -7672,8 +8863,35 @@
         <v>295.60000000000002</v>
       </c>
       <c r="K66" s="20"/>
-    </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M66" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="N66" s="20">
+        <v>39.6</v>
+      </c>
+      <c r="O66" s="20">
+        <v>30.7</v>
+      </c>
+      <c r="P66" s="20">
+        <v>30.4</v>
+      </c>
+      <c r="Q66" s="20">
+        <v>29</v>
+      </c>
+      <c r="R66" s="20">
+        <v>29.5</v>
+      </c>
+      <c r="S66" s="20">
+        <v>33.5</v>
+      </c>
+      <c r="T66" s="20">
+        <v>34</v>
+      </c>
+      <c r="U66" s="20">
+        <v>35.200000000000003</v>
+      </c>
+    </row>
+    <row r="67" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A67">
         <v>5</v>
       </c>
@@ -7705,8 +8923,35 @@
         <v>161.30000000000001</v>
       </c>
       <c r="K67" s="20"/>
-    </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M67" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="N67" s="20">
+        <v>42.4</v>
+      </c>
+      <c r="O67" s="20">
+        <v>29.4</v>
+      </c>
+      <c r="P67" s="20">
+        <v>29.5</v>
+      </c>
+      <c r="Q67" s="20">
+        <v>28.5</v>
+      </c>
+      <c r="R67" s="20">
+        <v>28.4</v>
+      </c>
+      <c r="S67" s="20">
+        <v>32.6</v>
+      </c>
+      <c r="T67" s="20">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="U67" s="20">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="68" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A68">
         <v>6</v>
       </c>
@@ -7738,8 +8983,35 @@
         <v>696.5</v>
       </c>
       <c r="K68" s="20"/>
-    </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M68" s="14" t="s">
+        <v>7</v>
+      </c>
+      <c r="N68" s="20">
+        <v>34.6</v>
+      </c>
+      <c r="O68" s="20">
+        <v>33.1</v>
+      </c>
+      <c r="P68" s="20">
+        <v>34.700000000000003</v>
+      </c>
+      <c r="Q68" s="20">
+        <v>34.5</v>
+      </c>
+      <c r="R68" s="20">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="S68" s="20">
+        <v>40.1</v>
+      </c>
+      <c r="T68" s="20">
+        <v>40.5</v>
+      </c>
+      <c r="U68" s="20">
+        <v>41.6</v>
+      </c>
+    </row>
+    <row r="69" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A69">
         <v>7</v>
       </c>
@@ -7771,8 +9043,35 @@
         <v>585.20000000000005</v>
       </c>
       <c r="K69" s="20"/>
-    </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M69" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="N69" s="20">
+        <v>22.8</v>
+      </c>
+      <c r="O69" s="20">
+        <v>17.8</v>
+      </c>
+      <c r="P69" s="20">
+        <v>14.3</v>
+      </c>
+      <c r="Q69" s="20">
+        <v>11.7</v>
+      </c>
+      <c r="R69" s="20">
+        <v>12.3</v>
+      </c>
+      <c r="S69" s="20">
+        <v>14.1</v>
+      </c>
+      <c r="T69" s="20">
+        <v>13.9</v>
+      </c>
+      <c r="U69" s="20">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="70" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A70">
         <v>8</v>
       </c>
@@ -7804,8 +9103,35 @@
         <v>201.6</v>
       </c>
       <c r="K70" s="20"/>
-    </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M70" s="14" t="s">
+        <v>9</v>
+      </c>
+      <c r="N70" s="20">
+        <v>47.4</v>
+      </c>
+      <c r="O70" s="20">
+        <v>36.4</v>
+      </c>
+      <c r="P70" s="20">
+        <v>37.4</v>
+      </c>
+      <c r="Q70" s="20">
+        <v>36.4</v>
+      </c>
+      <c r="R70" s="20">
+        <v>36.700000000000003</v>
+      </c>
+      <c r="S70" s="20">
+        <v>43.6</v>
+      </c>
+      <c r="T70" s="20">
+        <v>44.4</v>
+      </c>
+      <c r="U70" s="20">
+        <v>45.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A71">
         <v>9</v>
       </c>
@@ -7837,8 +9163,35 @@
         <v>99.3</v>
       </c>
       <c r="K71" s="20"/>
-    </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M71" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="N71" s="20">
+        <v>43.3</v>
+      </c>
+      <c r="O71" s="20">
+        <v>33.1</v>
+      </c>
+      <c r="P71" s="20">
+        <v>36.1</v>
+      </c>
+      <c r="Q71" s="20">
+        <v>33.700000000000003</v>
+      </c>
+      <c r="R71" s="20">
+        <v>35.9</v>
+      </c>
+      <c r="S71" s="20">
+        <v>42.5</v>
+      </c>
+      <c r="T71" s="20">
+        <v>43.5</v>
+      </c>
+      <c r="U71" s="20">
+        <v>44.9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A72">
         <v>10</v>
       </c>
@@ -7870,8 +9223,35 @@
         <v>153.1</v>
       </c>
       <c r="K72" s="20"/>
-    </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M72" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="N72" s="20">
+        <v>43.8</v>
+      </c>
+      <c r="O72" s="20">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="P72" s="20">
+        <v>35.6</v>
+      </c>
+      <c r="Q72" s="20">
+        <v>35.9</v>
+      </c>
+      <c r="R72" s="20">
+        <v>36.4</v>
+      </c>
+      <c r="S72" s="20">
+        <v>40.5</v>
+      </c>
+      <c r="T72" s="20">
+        <v>40.4</v>
+      </c>
+      <c r="U72" s="20">
+        <v>41.9</v>
+      </c>
+    </row>
+    <row r="73" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A73">
         <v>11</v>
       </c>
@@ -7903,8 +9283,35 @@
         <v>3040.8</v>
       </c>
       <c r="K73" s="20"/>
-    </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M73" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="N73" s="20">
+        <v>33.5</v>
+      </c>
+      <c r="O73" s="20">
+        <v>29.8</v>
+      </c>
+      <c r="P73" s="20">
+        <v>27.2</v>
+      </c>
+      <c r="Q73" s="20">
+        <v>28.1</v>
+      </c>
+      <c r="R73" s="20">
+        <v>28</v>
+      </c>
+      <c r="S73" s="20">
+        <v>31.7</v>
+      </c>
+      <c r="T73" s="20">
+        <v>31.3</v>
+      </c>
+      <c r="U73" s="20">
+        <v>32.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A74">
         <v>12</v>
       </c>
@@ -7936,8 +9343,35 @@
         <v>56.2</v>
       </c>
       <c r="K74" s="20"/>
-    </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M74" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="N74" s="20">
+        <v>34.5</v>
+      </c>
+      <c r="O74" s="20">
+        <v>26.8</v>
+      </c>
+      <c r="P74" s="20">
+        <v>25.1</v>
+      </c>
+      <c r="Q74" s="20">
+        <v>24</v>
+      </c>
+      <c r="R74" s="20">
+        <v>23.2</v>
+      </c>
+      <c r="S74" s="20">
+        <v>27.3</v>
+      </c>
+      <c r="T74" s="20">
+        <v>28.7</v>
+      </c>
+      <c r="U74" s="20">
+        <v>30.6</v>
+      </c>
+    </row>
+    <row r="75" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A75">
         <v>13</v>
       </c>
@@ -7969,23 +9403,108 @@
         <v>339.2</v>
       </c>
       <c r="K75" s="20"/>
-    </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+      <c r="M75" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="N75" s="20">
+        <v>45.8</v>
+      </c>
+      <c r="O75" s="20">
+        <v>36.299999999999997</v>
+      </c>
+      <c r="P75" s="20">
+        <v>38.299999999999997</v>
+      </c>
+      <c r="Q75" s="20">
+        <v>37.700000000000003</v>
+      </c>
+      <c r="R75" s="20">
+        <v>37.799999999999997</v>
+      </c>
+      <c r="S75" s="20">
+        <v>42.7</v>
+      </c>
+      <c r="T75" s="20">
+        <v>43.3</v>
+      </c>
+      <c r="U75" s="20">
+        <v>44.7</v>
+      </c>
+    </row>
+    <row r="76" spans="1:21" x14ac:dyDescent="0.2">
       <c r="J76">
         <f>SUM(J63:J75)</f>
         <v>6599.9</v>
       </c>
-      <c r="L76">
+      <c r="M76" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="N76" s="20">
+        <v>45.1</v>
+      </c>
+      <c r="O76" s="20">
+        <v>33.4</v>
+      </c>
+      <c r="P76" s="20">
+        <v>35.6</v>
+      </c>
+      <c r="Q76" s="20">
+        <v>34.5</v>
+      </c>
+      <c r="R76" s="20">
+        <v>33.799999999999997</v>
+      </c>
+      <c r="S76" s="20">
+        <v>37.200000000000003</v>
+      </c>
+      <c r="T76" s="20">
+        <v>38.6</v>
+      </c>
+      <c r="U76" s="20">
+        <v>40.299999999999997</v>
+      </c>
+    </row>
+    <row r="77" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="M77" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="N77" s="20">
+        <v>60.4</v>
+      </c>
+      <c r="O77" s="20">
+        <v>57.6</v>
+      </c>
+      <c r="P77" s="19">
+        <v>55.4</v>
+      </c>
+      <c r="Q77" s="19">
+        <v>56</v>
+      </c>
+      <c r="R77" s="19">
+        <v>54.8</v>
+      </c>
+      <c r="S77" s="19">
+        <v>57.3</v>
+      </c>
+      <c r="T77" s="19">
+        <v>61.4</v>
+      </c>
+      <c r="U77" s="23">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="80" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="I80">
         <f>J76/J58*100</f>
         <v>17.934608340262717</v>
       </c>
-      <c r="M76" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="M77" t="s">
-        <v>77</v>
+      <c r="J80" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="81" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="J81" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="82" spans="2:16" x14ac:dyDescent="0.2">
@@ -8238,7 +9757,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:3" ht="19" x14ac:dyDescent="0.25">
@@ -8266,6 +9785,11 @@
       </c>
       <c r="C3" s="2" t="s">
         <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C5" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>